<commit_message>
Tailor Excel research to user's brands (Kemppi premium, Sincosald)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HrHKPohdMvSwuBCcCr6jdL
</commit_message>
<xml_diff>
--- a/saldatrici-usate-buyer.xlsx
+++ b/saldatrici-usate-buyer.xlsx
@@ -1126,77 +1126,125 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">La marca decide il prezzo: premium (Miller, ESAB, Lincoln, Fronius, Cebora) = offerte buone; no-name = offerte basse.</t>
+          <t xml:space="preserve">La marca decide il prezzo: premium (Miller, ESAB, Lincoln, Fronius, Cebora, Kemppi) = offerte buone; no-name = offerte basse.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">TENSIONE / EXPORT</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le macchine italiane sono 230/400V 50Hz: si rivendono in UE (Westermans, Surplex, intermediari IT). I buyer USA (S.D. Nold, UWEL) vogliono 60Hz -&gt; non adatti.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">LE TUE MARCHE - Kemppi</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PREMIUM. Tra i marchi per cui i compratori pagano DI PIU sull'usato (insieme a ESAB, Fronius, Miller, Lincoln). Alta domanda in tutta Europa. Westermans ha una pagina dedicata all'acquisto/vendita di Kemppi MIG usate -&gt; per i lotti con Kemppi e il canale n.1 (prezzo migliore + ritiro UE).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AVVERTENZE</t>
+          <t xml:space="preserve">LE TUE MARCHE - Sincosald</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1) Verifica sempre i contatti prima di trattare (dati pubblici, possono cambiare). 2) Pagamento immediato = preferisci bonifico, mai anticipi/commissioni a carico tuo. 3) Per export verifica P.IVA/VIES e identita azienda.</t>
+          <t xml:space="preserve">Produttore italiano dal 1950 (NE Milano), qualita medio-alta (serie Evolution/Novamig). Si rivende bene in ITALIA: meglio gli intermediari italiani che conoscono il brand (Sigma, Eurosald). All'estero e meno riconosciuto -&gt; valore inferiore rispetto a Kemppi.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROSSIMO PASSO CONSIGLIATO</t>
+          <t xml:space="preserve">STRATEGIA PER MARCA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Per ogni operazione: prepara una scheda-lotto (marca, modello, n.serie, foto, stato), mandala a 2-3 buyer, prendi l'offerta migliore e usala come leva di vendita.</t>
+          <t xml:space="preserve">Lotti con Kemppi/ESAB/Miller -&gt; Westermans (export, paga di piu). Lotti con Sincosald/marche italiane -&gt; intermediari IT del Nord (Sigma/Eurosald). Meglio mandare a entrambi e confrontare le offerte.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">TENSIONE / EXPORT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Le macchine italiane sono 230/400V 50Hz: si rivendono in UE (Westermans, Surplex, intermediari IT). I buyer USA (S.D. Nold, UWEL) vogliono 60Hz -&gt; non adatti.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AVVERTENZE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1) Verifica sempre i contatti prima di trattare (dati pubblici, possono cambiare). 2) Pagamento immediato = preferisci bonifico, mai anticipi/commissioni a carico tuo. 3) Per export verifica P.IVA/VIES e identita azienda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROSSIMO PASSO CONSIGLIATO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Per ogni operazione: prepara una scheda-lotto (marca, modello, n.serie, foto, stato), mandala a 2-3 buyer, prendi l'offerta migliore e usala come leva di vendita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t xml:space="preserve">FONTI</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t xml:space="preserve">westermans.com/wanted.aspx; trustpilot.com/review/westermans.com; surplex.com; trustpilot/provenexpert Surplex; sigmainternational.it/usato; eurosald.com; salfershop.com/servizi; tecnogas-srl.it; sdnoldweldingsupplies.com + Birdeye; exapro.com; ebay/surplusrecord (prezzi MIG 300A)</t>
         </is>

</xml_diff>